<commit_message>
Stage 8.26A: polish Guided Match Lesson 1 teaching flow
Stage 8.26A: polish Guided Match Lesson 1 teaching flow
</commit_message>
<xml_diff>
--- a/ContentSource/Tutorial/FMCodex_Guided_Match.xlsx
+++ b/ContentSource/Tutorial/FMCodex_Guided_Match.xlsx
@@ -794,46 +794,46 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="GuideSteps" displayName="GuideSteps" ref="A1:L39" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" ns1:Ignorable="xr xr3" id="2" ns2:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="GuideSteps" displayName="GuideSteps" ref="A1:L41" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="LessonId"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="StepId"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="SurfaceType"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="TitleCN"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="BodyCN"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="SecondaryCN"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="CTA_CN"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="FocusTargetId"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="ArrowPlacement"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ShowExit"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="PointerCN"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0100-00000C000000}" name="Notes"/>
+    <tableColumn id="1" ns3:uid="{00000000-0010-0000-0100-000001000000}" name="LessonId"/>
+    <tableColumn id="2" ns3:uid="{00000000-0010-0000-0100-000002000000}" name="StepId"/>
+    <tableColumn id="3" ns3:uid="{00000000-0010-0000-0100-000003000000}" name="SurfaceType"/>
+    <tableColumn id="4" ns3:uid="{00000000-0010-0000-0100-000004000000}" name="TitleCN"/>
+    <tableColumn id="5" ns3:uid="{00000000-0010-0000-0100-000005000000}" name="BodyCN"/>
+    <tableColumn id="6" ns3:uid="{00000000-0010-0000-0100-000006000000}" name="SecondaryCN"/>
+    <tableColumn id="7" ns3:uid="{00000000-0010-0000-0100-000007000000}" name="CTA_CN"/>
+    <tableColumn id="8" ns3:uid="{00000000-0010-0000-0100-000008000000}" name="FocusTargetId"/>
+    <tableColumn id="9" ns3:uid="{00000000-0010-0000-0100-000009000000}" name="ArrowPlacement"/>
+    <tableColumn id="10" ns3:uid="{00000000-0010-0000-0100-00000A000000}" name="ShowExit"/>
+    <tableColumn id="11" ns3:uid="{00000000-0010-0000-0100-00000B000000}" name="PointerCN"/>
+    <tableColumn id="12" ns3:uid="{00000000-0010-0000-0100-00000C000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="GuideEmphasis" displayName="GuideEmphasis" ref="A1:F42" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" ns1:Ignorable="xr xr3" id="3" ns2:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="GuideEmphasis" displayName="GuideEmphasis" ref="A1:F48" totalsRowShown="0">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="LessonId"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="StepId"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Field"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="MatchText"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Occurrence"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Style"/>
+    <tableColumn id="1" ns3:uid="{00000000-0010-0000-0200-000001000000}" name="LessonId"/>
+    <tableColumn id="2" ns3:uid="{00000000-0010-0000-0200-000002000000}" name="StepId"/>
+    <tableColumn id="3" ns3:uid="{00000000-0010-0000-0200-000003000000}" name="Field"/>
+    <tableColumn id="4" ns3:uid="{00000000-0010-0000-0200-000004000000}" name="MatchText"/>
+    <tableColumn id="5" ns3:uid="{00000000-0010-0000-0200-000005000000}" name="Occurrence"/>
+    <tableColumn id="6" ns3:uid="{00000000-0010-0000-0200-000006000000}" name="Style"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="GuideTimings" displayName="GuideTimings" ref="A1:D16" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" ns1:Ignorable="xr xr3" id="4" ns2:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="GuideTimings" displayName="GuideTimings" ref="A1:D17" totalsRowShown="0">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="LessonId"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="TimingId"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Value"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Notes"/>
+    <tableColumn id="1" ns3:uid="{00000000-0010-0000-0300-000001000000}" name="LessonId"/>
+    <tableColumn id="2" ns3:uid="{00000000-0010-0000-0300-000002000000}" name="TimingId"/>
+    <tableColumn id="3" ns3:uid="{00000000-0010-0000-0300-000003000000}" name="Value"/>
+    <tableColumn id="4" ns3:uid="{00000000-0010-0000-0300-000004000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1112,11 +1112,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF6696B1"/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1241,18 +1241,24 @@
       <c r="C4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>34</v>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">确认进攻战术点</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">本回合进攻战术点为 {CurrentAttackTP}。请将鼠标移至左上角高亮的战术点数值处查看。进攻战术点决定本回合持球球员可以使用哪些技能。</t>
+        </is>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>24</v>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header.AttackTacticalPoint</t>
+        </is>
       </c>
       <c r="I4" s="1" t="s">
         <v>25</v>
@@ -1261,7 +1267,11 @@
         <v>1</v>
       </c>
       <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">先观察真实 HUD 数值，再点击继续；战术点匹配技能范围，不是普通球员部署资格。</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="62.1" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -1273,8 +1283,10 @@
       <c r="C5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>37</v>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">观察球员技能</t>
+        </is>
       </c>
       <c r="E5" s="4" t="s">
         <v>38</v>
@@ -1303,11 +1315,15 @@
       <c r="C6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>41</v>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">换个人，观察特性</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">这次换{ComparisonCarrier.DisplayName}试试。鼠标移至本方球员区的{ComparisonCarrier.DisplayName}处悬停，查看他的特性。</t>
+        </is>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="1"/>
@@ -1353,7 +1369,11 @@
         <v>1</v>
       </c>
       <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">保留稳定 ID；Lesson 1 两轮均不进入这个独立属性讲解步骤。</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="81" customHeight="1">
       <c r="A8" s="1" t="s">
@@ -2349,16 +2369,116 @@
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
     </row>
+    <row r="40" spans="1:12" ht="62.1" customHeight="1">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaHover.Comparison</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CompactActionBar</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">数值来源</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">鼠标移至进攻公式中的 {Formula.AttackBaseValue}，查看数值来源。</t>
+        </is>
+      </c>
+      <c r="F40" s="4"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formula.AttackBaseValue</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">第二次进攻掷骰前，观察真实生产公式 tooltip。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="84.95" customHeight="1">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaExplanation.Comparison</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ExplanationPanel</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">特性如何影响公式</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{ComparisonCarrier.DisplayName}的射门属性为 {Formula.AttackShooting}，{LongShot.TraitName}额外提供 +{Formula.AttackTraitBonus}，因此进攻基础值为 {Formula.AttackBaseValue}。</t>
+        </is>
+      </c>
+      <c r="F41" s="4"/>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">继续</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formula.AttackBaseValue</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">三个数值均只读当前权威 FormulaFacts，不在教学中相加。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" sqref="C2:C39" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" sqref="C2:C41" ns2:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"ExplanationPanel,CompactActionBar"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="I2:I39" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="I2:I41" ns2:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Auto,Above,Side,None"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="J2:J39" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" sqref="J2:J41" ns2:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2370,11 +2490,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF6696B1"/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -2674,8 +2794,10 @@
       <c r="C15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>152</v>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">特性</t>
+        </is>
       </c>
       <c r="E15" s="1">
         <v>1</v>
@@ -3222,15 +3344,195 @@
       </c>
       <c r="F42" s="1" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TacticPointExplanation</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TitleCN</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进攻战术点</t>
+        </is>
+      </c>
+      <c r="E43" s="1">
+        <v>1</v>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaHover.Comparison</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BodyCN</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{Formula.AttackBaseValue}</t>
+        </is>
+      </c>
+      <c r="E44" s="1">
+        <v>1</v>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaExplanation.Comparison</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TitleCN</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">特性</t>
+        </is>
+      </c>
+      <c r="E45" s="1">
+        <v>1</v>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaExplanation.Comparison</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BodyCN</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">射门属性</t>
+        </is>
+      </c>
+      <c r="E46" s="1">
+        <v>1</v>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaExplanation.Comparison</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BodyCN</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{LongShot.TraitName}</t>
+        </is>
+      </c>
+      <c r="E47" s="1">
+        <v>1</v>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="45.95" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FormulaExplanation.Comparison</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BodyCN</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">进攻基础值</t>
+        </is>
+      </c>
+      <c r="E48" s="1">
+        <v>1</v>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PerGlyphDots</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C2:C42" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="C2:C48" ns2:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"TitleCN,BodyCN"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="F2:F42" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" sqref="F2:F48" ns2:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"PerGlyphDots"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3242,11 +3544,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF6696B1"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -3477,6 +3779,26 @@
       </c>
       <c r="D16" s="1" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="45.95" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson01</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FullCardExplanationDelay</t>
+        </is>
+      </c>
+      <c r="C17" s="5">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">秒；真实 Full Card 可见后计时，离开卡牌或退出确认立即取消；仅用于两次卡牌检查。</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stage 8.27A: consolidate traits and refresh player content and Lesson 1
Stage 8.27A: consolidate traits and refresh player content and Lesson 1
</commit_message>
<xml_diff>
--- a/ContentSource/Tutorial/FMCodex_Guided_Match.xlsx
+++ b/ContentSource/Tutorial/FMCodex_Guided_Match.xlsx
@@ -1277,8 +1277,10 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>36</v>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>InspectRice</t>
+        </is>
       </c>
       <c r="C5" s="1" t="s">
         <v>27</v>
@@ -1420,8 +1422,10 @@
       <c r="D9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>52</v>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>{ComparisonCarrier.DisplayName}拥有「{LongShot.TraitName}」。直接远射时，这项特性提供射门 +1。</t>
+        </is>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="1" t="s">
@@ -1702,8 +1706,10 @@
       <c r="D18" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>81</v>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>对方安排门将参与本次防守，然后结束部署。</t>
+        </is>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="1"/>
@@ -2041,7 +2047,11 @@
       <c r="E29" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="F29" s="4"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>两次进攻使用相同防守阵容和骰点；防守公式包含门将参与加成。</t>
+        </is>
+      </c>
       <c r="G29" s="1" t="s">
         <v>35</v>
       </c>
@@ -2285,8 +2295,10 @@
       <c r="E37" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F37" s="4" t="s">
-        <v>139</v>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>本次对照中，{LongShot.TraitName} 提供了射门 +1。正式比赛中，结果仍会受到骰点和对手配置影响。</t>
+        </is>
       </c>
       <c r="G37" s="1" t="s">
         <v>140</v>
@@ -2319,8 +2331,10 @@
       <c r="E38" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F38" s="4" t="s">
-        <v>139</v>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>本次对照中，{LongShot.TraitName} 提供了射门 +1。正式比赛中，结果仍会受到骰点和对手配置影响。</t>
+        </is>
       </c>
       <c r="G38" s="1" t="s">
         <v>140</v>
@@ -2768,8 +2782,10 @@
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>36</v>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>InspectRice</t>
+        </is>
       </c>
       <c r="C14" s="1" t="s">
         <v>12</v>

</xml_diff>